<commit_message>
docs: cenário enxuto de ferramentas (planos gratuitos e bot de WhatsApp próprio)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018P8tNa7TjbnCtoUzBLkSAJ
</commit_message>
<xml_diff>
--- a/docs/negocio/Guinchei-Custos-MVP.xlsx
+++ b/docs/negocio/Guinchei-Custos-MVP.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="189">
   <si>
     <t xml:space="preserve">Premissas</t>
   </si>
@@ -115,6 +115,18 @@
     <t xml:space="preserve">Implícito nos documentos (R$ 51 líquido − R$ 48 de contribuição madura); associado a suporte e Disputa</t>
   </si>
   <si>
+    <t xml:space="preserve">Número de WhatsApp dedicado (chip), R$/mês ⚠️</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimativa: número comprado para o bot de login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hospedagem do bot de mensagens, R$/mês ⚠️</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 se rodar em servidor/n8n já existente; ~R$ 30 em VPS pequena</t>
+  </si>
+  <si>
     <t xml:space="preserve">Investimento do MVP (6 meses)</t>
   </si>
   <si>
@@ -133,6 +145,9 @@
     <t xml:space="preserve">% do total</t>
   </si>
   <si>
+    <t xml:space="preserve">Cenário enxuto (R$)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Desenvolvimento do PWA (3 superfícies)</t>
   </si>
   <si>
@@ -181,6 +196,9 @@
     <t xml:space="preserve">Subsídio por Frota por mês</t>
   </si>
   <si>
+    <t xml:space="preserve">Economia do cenário enxuto vs. base</t>
+  </si>
+  <si>
     <t xml:space="preserve">Por grupo</t>
   </si>
   <si>
@@ -196,10 +214,10 @@
     <t xml:space="preserve">Tecnologia</t>
   </si>
   <si>
-    <t xml:space="preserve">Mínimo/mês (R$)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Máximo/mês (R$)</t>
+    <t xml:space="preserve">Enxuto/mês (R$): planos grátis + bot próprio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Escala/mês (R$): planos pagos + API oficial</t>
   </si>
   <si>
     <t xml:space="preserve">Observação</t>
@@ -220,7 +238,7 @@
     <t xml:space="preserve">Vercel</t>
   </si>
   <si>
-    <t xml:space="preserve">Mín.: Hobby (grátis). Máx.: Pro, US$ 20</t>
+    <t xml:space="preserve">Enxuto: Hobby (grátis; uso não comercial). Escala: Pro, US$ 20</t>
   </si>
   <si>
     <t xml:space="preserve">Back-end</t>
@@ -229,7 +247,7 @@
     <t xml:space="preserve">Supabase (Postgres+PostGIS, Auth, Storage, Realtime)</t>
   </si>
   <si>
-    <t xml:space="preserve">Mín.: Free. Máx.: Pro, US$ 25</t>
+    <t xml:space="preserve">Enxuto: Free (pausa por inatividade, sem backup). Escala: Pro, US$ 25</t>
   </si>
   <si>
     <t xml:space="preserve">Mapas, geocoding e rotas</t>
@@ -241,13 +259,13 @@
     <t xml:space="preserve">Cota gratuita; cobra por uso acima dela</t>
   </si>
   <si>
-    <t xml:space="preserve">Login por telefone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WhatsApp/SMS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Códigos/mês × custo por código</t>
+    <t xml:space="preserve">Login por telefone (código por WhatsApp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enxuto: número próprio + bot (ex.: n8n). Escala: API oficial do WhatsApp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enxuto: chip + hospedagem do bot. Escala: códigos/mês × custo por código. Bot não oficial pode ser banido pelo WhatsApp</t>
   </si>
   <si>
     <t xml:space="preserve">Domínio .com.br</t>
@@ -648,15 +666,15 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
       <sz val="10"/>
+      <color rgb="FF008000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
       <sz val="10"/>
-      <color rgb="FF008000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -794,7 +812,15 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -802,15 +828,15 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -818,10 +844,6 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -830,7 +852,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -838,11 +860,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -854,11 +872,11 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1118,7 +1136,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
@@ -1321,6 +1339,28 @@
       </c>
       <c r="C20" s="7" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1339,45 +1379,49 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>34</v>
+        <v>38</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>0</v>
@@ -1386,13 +1430,17 @@
         <f aca="false">C5/$C$13</f>
         <v>0</v>
       </c>
+      <c r="E5" s="14" t="n">
+        <f aca="false">C5</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>7000</v>
@@ -1401,13 +1449,17 @@
         <f aca="false">C6/$C$13</f>
         <v>0.107692307692308</v>
       </c>
+      <c r="E6" s="15" t="n">
+        <f aca="false">Stack!C14</f>
+        <v>260</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>5000</v>
@@ -1416,13 +1468,17 @@
         <f aca="false">C7/$C$13</f>
         <v>0.0769230769230769</v>
       </c>
+      <c r="E7" s="14" t="n">
+        <f aca="false">C7</f>
+        <v>5000</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>6000</v>
@@ -1431,13 +1487,17 @@
         <f aca="false">C8/$C$13</f>
         <v>0.0923076923076923</v>
       </c>
+      <c r="E8" s="14" t="n">
+        <f aca="false">C8</f>
+        <v>6000</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>9000</v>
@@ -1446,13 +1506,17 @@
         <f aca="false">C9/$C$13</f>
         <v>0.138461538461538</v>
       </c>
+      <c r="E9" s="14" t="n">
+        <f aca="false">C9</f>
+        <v>9000</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>43</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>38</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>18000</v>
@@ -1461,13 +1525,17 @@
         <f aca="false">C10/$C$13</f>
         <v>0.276923076923077</v>
       </c>
+      <c r="E10" s="14" t="n">
+        <f aca="false">C10</f>
+        <v>18000</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="C11" s="6" t="n">
         <v>12000</v>
@@ -1476,13 +1544,17 @@
         <f aca="false">C11/$C$13</f>
         <v>0.184615384615385</v>
       </c>
+      <c r="E11" s="14" t="n">
+        <f aca="false">C11</f>
+        <v>12000</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>8000</v>
@@ -1491,57 +1563,74 @@
         <f aca="false">C12/$C$13</f>
         <v>0.123076923076923</v>
       </c>
+      <c r="E12" s="14" t="n">
+        <f aca="false">C12</f>
+        <v>8000</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="16" t="n">
+      <c r="A13" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13" s="17"/>
+      <c r="C13" s="18" t="n">
         <f aca="false">SUM(C5:C12)</f>
         <v>65000</v>
       </c>
-      <c r="D13" s="17" t="n">
+      <c r="D13" s="19" t="n">
         <f aca="false">SUM(D5:D12)</f>
         <v>1</v>
       </c>
+      <c r="E13" s="18" t="n">
+        <f aca="false">SUM(E5:E12)</f>
+        <v>58260</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="C15" s="19" t="n">
+      <c r="A15" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="C15" s="15" t="n">
         <f aca="false">C13/Premissas!B9</f>
         <v>10833.3333333333</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="C16" s="19" t="n">
+        <v>55</v>
+      </c>
+      <c r="C16" s="15" t="n">
         <f aca="false">C10/Premissas!B15/Premissas!B16</f>
         <v>2000</v>
       </c>
     </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E17" s="21" t="n">
+        <f aca="false">C13-E13</f>
+        <v>6740</v>
+      </c>
+    </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B19" s="5"/>
-      <c r="C19" s="20" t="n">
+      <c r="C19" s="14" t="n">
         <f aca="false">SUMIF($B$5:$B$12,A19,$C$5:$C$12)</f>
         <v>20000</v>
       </c>
@@ -1552,10 +1641,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B20" s="5"/>
-      <c r="C20" s="20" t="n">
+      <c r="C20" s="14" t="n">
         <f aca="false">SUMIF($B$5:$B$12,A20,$C$5:$C$12)</f>
         <v>25000</v>
       </c>
@@ -1566,10 +1655,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B21" s="5"/>
-      <c r="C21" s="20" t="n">
+      <c r="C21" s="14" t="n">
         <f aca="false">SUMIF($B$5:$B$12,A21,$C$5:$C$12)</f>
         <v>12000</v>
       </c>
@@ -1580,10 +1669,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B22" s="5"/>
-      <c r="C22" s="20" t="n">
+      <c r="C22" s="14" t="n">
         <f aca="false">SUMIF($B$5:$B$12,A22,$C$5:$C$12)</f>
         <v>8000</v>
       </c>
@@ -1594,10 +1683,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B23" s="5"/>
-      <c r="C23" s="20" t="n">
+      <c r="C23" s="14" t="n">
         <f aca="false">SUMIF($B$5:$B$12,A23,$C$5:$C$12)</f>
         <v>0</v>
       </c>
@@ -1633,226 +1722,226 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="C5" s="21" t="n">
+        <v>66</v>
+      </c>
+      <c r="C5" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D5" s="21" t="n">
+      <c r="D5" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="22" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E5" s="23" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="C6" s="21" t="n">
+        <v>69</v>
+      </c>
+      <c r="C6" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="23" t="n">
+      <c r="D6" s="24" t="n">
         <f aca="false">20*Premissas!B12</f>
         <v>110</v>
       </c>
-      <c r="E6" s="22" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E6" s="23" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="C7" s="21" t="n">
+        <v>72</v>
+      </c>
+      <c r="C7" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="23" t="n">
+      <c r="D7" s="24" t="n">
         <f aca="false">25*Premissas!B12</f>
         <v>137.5</v>
       </c>
-      <c r="E7" s="22" t="s">
-        <v>67</v>
+      <c r="E7" s="23" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="C8" s="21" t="n">
+        <v>75</v>
+      </c>
+      <c r="C8" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="21" t="n">
+      <c r="D8" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="22" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E8" s="23" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="C9" s="23" t="n">
+        <v>78</v>
+      </c>
+      <c r="C9" s="24" t="n">
+        <f aca="false">Premissas!B21+Premissas!B22</f>
+        <v>40</v>
+      </c>
+      <c r="D9" s="24" t="n">
         <f aca="false">Premissas!B13*Premissas!B14</f>
         <v>240</v>
       </c>
-      <c r="D9" s="23" t="n">
-        <f aca="false">Premissas!B13*Premissas!B14</f>
-        <v>240</v>
-      </c>
-      <c r="E9" s="22" t="s">
-        <v>73</v>
+      <c r="E9" s="23" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="C10" s="24" t="n">
+        <v>81</v>
+      </c>
+      <c r="C10" s="25" t="n">
         <f aca="false">40/12</f>
         <v>3.33333333333333</v>
       </c>
-      <c r="D10" s="24" t="n">
+      <c r="D10" s="25" t="n">
         <f aca="false">40/12</f>
         <v>3.33333333333333</v>
       </c>
-      <c r="E10" s="22" t="s">
-        <v>76</v>
+      <c r="E10" s="23" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="C11" s="21" t="n">
+        <v>84</v>
+      </c>
+      <c r="C11" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="21" t="n">
+      <c r="D11" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="22" t="s">
-        <v>79</v>
+      <c r="E11" s="23" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="C12" s="21" t="n">
+        <v>87</v>
+      </c>
+      <c r="C12" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="21" t="n">
+      <c r="D12" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="22" t="s">
-        <v>82</v>
+      <c r="E12" s="23" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="25" t="n">
+      <c r="A13" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="B13" s="17"/>
+      <c r="C13" s="26" t="n">
         <f aca="false">SUM(C5:C12)</f>
-        <v>243.333333333333</v>
-      </c>
-      <c r="D13" s="25" t="n">
+        <v>43.3333333333333</v>
+      </c>
+      <c r="D13" s="26" t="n">
         <f aca="false">SUM(D5:D12)</f>
         <v>490.833333333333</v>
       </c>
-      <c r="E13" s="15"/>
+      <c r="E13" s="17"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="B14" s="5"/>
-      <c r="C14" s="19" t="n">
+      <c r="C14" s="15" t="n">
         <f aca="false">C13*Premissas!B9</f>
-        <v>1460</v>
-      </c>
-      <c r="D14" s="19" t="n">
+        <v>260</v>
+      </c>
+      <c r="D14" s="15" t="n">
         <f aca="false">D13*Premissas!B9</f>
         <v>2945</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="B15" s="5"/>
-      <c r="C15" s="19" t="n">
+      <c r="C15" s="15" t="n">
         <f aca="false">Investimento!C6</f>
         <v>7000</v>
       </c>
-      <c r="D15" s="19" t="n">
+      <c r="D15" s="15" t="n">
         <f aca="false">Investimento!C6</f>
         <v>7000</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="18" t="s">
-        <v>86</v>
+      <c r="A16" s="20" t="s">
+        <v>92</v>
       </c>
       <c r="B16" s="5"/>
-      <c r="C16" s="26" t="n">
+      <c r="C16" s="21" t="n">
         <f aca="false">C15-C14</f>
-        <v>5540</v>
-      </c>
-      <c r="D16" s="26" t="n">
+        <v>6740</v>
+      </c>
+      <c r="D16" s="21" t="n">
         <f aca="false">D15-D14</f>
         <v>4055</v>
       </c>
@@ -1884,109 +1973,109 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="27" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="D5" s="19" t="n">
+        <v>102</v>
+      </c>
+      <c r="D5" s="15" t="n">
         <f aca="false">Investimento!C7</f>
         <v>5000</v>
       </c>
-      <c r="E5" s="19" t="n">
+      <c r="E5" s="15" t="n">
         <f aca="false">Investimento!C7</f>
         <v>5000</v>
       </c>
-      <c r="F5" s="22" t="s">
-        <v>97</v>
+      <c r="F5" s="23" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="27" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="D6" s="19" t="n">
+        <v>102</v>
+      </c>
+      <c r="D6" s="15" t="n">
         <f aca="false">Investimento!C8</f>
         <v>6000</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="15" t="n">
         <f aca="false">Investimento!C8</f>
         <v>6000</v>
       </c>
-      <c r="F6" s="22" t="s">
-        <v>97</v>
+      <c r="F6" s="23" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="D7" s="19" t="n">
+        <v>102</v>
+      </c>
+      <c r="D7" s="15" t="n">
         <f aca="false">Investimento!C9</f>
         <v>9000</v>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="15" t="n">
         <f aca="false">Investimento!C9</f>
         <v>9000</v>
       </c>
-      <c r="F7" s="22" t="s">
-        <v>97</v>
+      <c r="F7" s="23" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="27" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>0</v>
@@ -1994,19 +2083,19 @@
       <c r="E8" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="22" t="s">
-        <v>105</v>
+      <c r="F8" s="23" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>0</v>
@@ -2014,19 +2103,19 @@
       <c r="E9" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="22" t="s">
-        <v>108</v>
+      <c r="F9" s="23" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="27" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B10" s="27" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D10" s="6" t="n">
         <v>0</v>
@@ -2034,19 +2123,19 @@
       <c r="E10" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="22" t="s">
-        <v>111</v>
+      <c r="F10" s="23" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D11" s="6" t="n">
         <v>0</v>
@@ -2054,19 +2143,19 @@
       <c r="E11" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="22" t="s">
-        <v>114</v>
+      <c r="F11" s="23" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="27" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B12" s="27" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D12" s="12" t="n">
         <v>400</v>
@@ -2074,33 +2163,33 @@
       <c r="E12" s="12" t="n">
         <v>700</v>
       </c>
-      <c r="F12" s="22" t="s">
-        <v>117</v>
+      <c r="F12" s="23" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="16" t="n">
+      <c r="A13" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="18" t="n">
         <f aca="false">SUMIF($C$5:$C$12,"Plataforma",D5:D12)</f>
         <v>20400</v>
       </c>
-      <c r="E13" s="16" t="n">
+      <c r="E13" s="18" t="n">
         <f aca="false">SUMIF($C$5:$C$12,"Plataforma",E5:E12)</f>
         <v>20700</v>
       </c>
-      <c r="F13" s="15"/>
+      <c r="F13" s="17"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B14" s="5"/>
       <c r="C14" s="5" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D14" s="12" t="n">
         <v>400</v>
@@ -2109,7 +2198,7 @@
         <v>800</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -2138,78 +2227,78 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="B5" s="19" t="n">
+        <v>131</v>
+      </c>
+      <c r="B5" s="15" t="n">
         <f aca="false">Premissas!B5</f>
         <v>300</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="20" t="n">
+      <c r="B6" s="14" t="n">
         <f aca="false">B5*Premissas!B6</f>
         <v>60</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="B7" s="20" t="n">
+        <v>134</v>
+      </c>
+      <c r="B7" s="14" t="n">
         <f aca="false">B5-B6</f>
         <v>240</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="B8" s="20" t="n">
+        <v>136</v>
+      </c>
+      <c r="B8" s="14" t="n">
         <f aca="false">-B5*Premissas!B7</f>
         <v>-9</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="B9" s="16" t="n">
+      <c r="A9" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="B9" s="18" t="n">
         <f aca="false">B6+B8</f>
         <v>51</v>
       </c>
@@ -2217,38 +2306,38 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="B10" s="20" t="n">
+        <v>139</v>
+      </c>
+      <c r="B10" s="14" t="n">
         <f aca="false">-Premissas!B8</f>
         <v>-25</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="B11" s="16" t="n">
+      <c r="A11" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="B11" s="18" t="n">
         <f aca="false">B9+B10</f>
         <v>26</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="B12" s="16" t="n">
+      <c r="A12" s="16" t="s">
+        <v>143</v>
+      </c>
+      <c r="B12" s="18" t="n">
         <f aca="false">B9-Premissas!B20</f>
         <v>48</v>
       </c>
       <c r="C12" s="28" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -2277,37 +2366,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="B5" s="19" t="n">
+        <v>151</v>
+      </c>
+      <c r="B5" s="15" t="n">
         <f aca="false">Premissas!B10</f>
         <v>5500</v>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="C5" s="15" t="n">
         <f aca="false">'Unit economics'!B11</f>
         <v>26</v>
       </c>
@@ -2318,13 +2407,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="B6" s="19" t="n">
+        <v>152</v>
+      </c>
+      <c r="B6" s="15" t="n">
         <f aca="false">Premissas!B10</f>
         <v>5500</v>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="15" t="n">
         <f aca="false">'Unit economics'!B12</f>
         <v>48</v>
       </c>
@@ -2335,13 +2424,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="B7" s="19" t="n">
+        <v>153</v>
+      </c>
+      <c r="B7" s="15" t="n">
         <f aca="false">Premissas!B11</f>
         <v>18000</v>
       </c>
-      <c r="C7" s="19" t="n">
+      <c r="C7" s="15" t="n">
         <f aca="false">'Unit economics'!B12</f>
         <v>48</v>
       </c>
@@ -2352,21 +2441,21 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B11" s="30" t="n">
         <f aca="false">Premissas!B17</f>
@@ -2383,41 +2472,41 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="B12" s="20" t="n">
+        <v>159</v>
+      </c>
+      <c r="B12" s="14" t="n">
         <f aca="false">B11*Premissas!$B$5</f>
         <v>90000</v>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="14" t="n">
         <f aca="false">C11*Premissas!$B$5</f>
         <v>120000</v>
       </c>
-      <c r="D12" s="20" t="n">
+      <c r="D12" s="14" t="n">
         <f aca="false">D11*Premissas!$B$5</f>
         <v>150000</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="B13" s="20" t="n">
+        <v>160</v>
+      </c>
+      <c r="B13" s="14" t="n">
         <f aca="false">B12*Premissas!$B$6</f>
         <v>18000</v>
       </c>
-      <c r="C13" s="20" t="n">
+      <c r="C13" s="14" t="n">
         <f aca="false">C12*Premissas!$B$6</f>
         <v>24000</v>
       </c>
-      <c r="D13" s="20" t="n">
+      <c r="D13" s="14" t="n">
         <f aca="false">D12*Premissas!$B$6</f>
         <v>30000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>3</v>
@@ -2427,7 +2516,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="B16" s="30" t="n">
         <f aca="false">Premissas!B19</f>
@@ -2436,36 +2525,36 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="B17" s="20" t="n">
+        <v>163</v>
+      </c>
+      <c r="B17" s="14" t="n">
         <f aca="false">B16*Premissas!B5</f>
         <v>450000</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="B18" s="20" t="n">
+        <v>164</v>
+      </c>
+      <c r="B18" s="14" t="n">
         <f aca="false">B17*Premissas!B6</f>
         <v>90000</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
-        <v>159</v>
-      </c>
-      <c r="B19" s="16" t="n">
+      <c r="A19" s="16" t="s">
+        <v>165</v>
+      </c>
+      <c r="B19" s="18" t="n">
         <f aca="false">B16*'Unit economics'!B12</f>
         <v>72000</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="B20" s="20" t="n">
+        <v>166</v>
+      </c>
+      <c r="B20" s="14" t="n">
         <f aca="false">B19-Premissas!B11</f>
         <v>54000</v>
       </c>
@@ -2497,12 +2586,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2510,75 +2599,75 @@
         <v>4</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>168</v>
-      </c>
-      <c r="D5" s="19" t="n">
+        <v>174</v>
+      </c>
+      <c r="D5" s="15" t="n">
         <f aca="false">'Unit economics'!B6</f>
         <v>60</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -2586,22 +2675,22 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>

</xml_diff>